<commit_message>
Finalize D1 floor Step calibration and PLS peers
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_mapping_params.xlsx
+++ b/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_mapping_params.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mapping_master" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mapping_versions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mapping_examples" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="step_calibration_summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,6 +512,16 @@
           <t>window_scope</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>calibration_id</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>calibration_scope</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -579,6 +590,8 @@
           <t>6h</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -612,35 +625,45 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>v1.1</t>
+          <t>1.3.0-final-candidate</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>expert_calibrated</t>
+          <t>detector_input_fault_injection</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>DO/ORP only</t>
+          <t>iid-routed DO/ORP mapping domain; other routes audited separately</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>24h</t>
+          <t>24h main + 36h confirmation</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>step-injection-ea8d55282211</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>iid routed inputs; 780 sustained-step scenarios; 10-channel LOCO</t>
         </is>
       </c>
     </row>
@@ -707,6 +730,8 @@
           <t>168h main</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -775,6 +800,8 @@
           <t>6h main</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -839,6 +866,8 @@
           <t>6h main</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -903,6 +932,8 @@
           <t>6h main</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -967,6 +998,8 @@
           <t>336h main</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1072,7 +1105,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1080,7 +1113,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>causal six-state recovery + event-level validation; mapping coefficients unchanged</t>
+          <t>causal recovery + event validation + raw-input Step fault injection; step-injection-ea8d55282211</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1125,7 +1158,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>4.84</v>
+        <v>4.999397158567762</v>
       </c>
     </row>
     <row r="3">
@@ -1135,10 +1168,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="C3" t="n">
-        <v>4.33</v>
+        <v>4.96734971538736</v>
       </c>
     </row>
     <row r="4">
@@ -1148,10 +1181,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="C4" t="n">
-        <v>3.76</v>
+        <v>4.667309214024311</v>
       </c>
     </row>
     <row r="5">
@@ -1161,7 +1194,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="C5" t="n">
         <v>3</v>
@@ -1170,27 +1203,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>D1_drift</t>
+          <t>D1_step</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="C6" t="n">
-        <v>4.62</v>
+        <v>1.33269078597569</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D1_drift</t>
+          <t>D1_step</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>1.002984115335347</v>
       </c>
     </row>
     <row r="8">
@@ -1200,36 +1233,36 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>1.38</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>D1_regime</t>
+          <t>D1_drift</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="C9" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>D1_regime</t>
+          <t>D1_drift</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="11">
@@ -1239,10 +1272,160 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>D1_regime</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>D1_regime</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>5</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C13" t="n">
         <v>1.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>calibration_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>library_sha256</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>selected_k</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>selected_x0</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>rmse_channel_balanced</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>null_warning_rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>small_hard_rate</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>material_detection_rate</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>material_miss_rate</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>source_run_id</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>included_scoring_modes</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>excluded_scoring_modes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>step-injection-ea8d55282211</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>775d423be3d728fd48533c6e84bfc07af3233164dc6186bf33b3c1969259b970</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.6712747728961548</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.008333333333333333</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>d1-final-57bdbc83894f</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>iid</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>autocorr_aware;floor_freeze</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>